<commit_message>
updates trap data and metadata, updates project metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata/lower_feather_trap_metadata.xlsx
+++ b/data-raw/metadata/lower_feather_trap_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-lower-feather-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9EBDEA-5239-4AC5-AE53-982B948F9E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E0B2E3-580E-4222-9D23-7ED60451FB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="680" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9380" yWindow="350" windowWidth="16220" windowHeight="14180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -268,10 +268,10 @@
     <t xml:space="preserve"> End date and time of a trapping period. Derived from visitTime and visitTime2 fields, adjusted based on the visitType field</t>
   </si>
   <si>
-    <t>2026-01-27 10:00:58</t>
+    <t>2026-02-13 10:30:58</t>
   </si>
   <si>
-    <t>2026-01-26 10:00:41</t>
+    <t>2026-02-12 10:30:58</t>
   </si>
 </sst>
 </file>

</xml_diff>